<commit_message>
refactor: organize products into self-contained families
Move each product into a single family-scoped folder, update portfolio paths and references, retain product-local history and dependencies, and add layout validation and migration documentation.
</commit_message>
<xml_diff>
--- a/business/02-portfolio/product-portfolio.xlsx
+++ b/business/02-portfolio/product-portfolio.xlsx
@@ -258,7 +258,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
@@ -273,7 +273,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -288,7 +288,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
@@ -1620,14 +1620,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="31" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="33" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
@@ -1643,6 +1643,9 @@
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="48" customWidth="1"/>
     <col min="20" max="20" width="48" customWidth="1"/>
+    <col min="21" max="21" width="46" customWidth="1"/>
+    <col min="22" max="22" width="48" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1746,6 +1749,21 @@
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model_Status</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model_Evidence_Path</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model_Audit_Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1848,6 +1866,21 @@
           <t xml:space="preserve">Do not call exact-fit or IKEA-compatible until the named drawer revision and measurement tolerance are physically proven</t>
         </is>
       </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">organizer/drawer-inlay/DRAFT-schubladen-organizer-R1.3-aspect-safe-030mm/schubladen-organizer/output/DRAFT/DRAFT-R1.3-aspect-safe-030mm-assembly.3mf</t>
+        </is>
+      </c>
+      <c r="W2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1950,6 +1983,21 @@
           <t xml:space="preserve">DRAFT digital candidate only; estimated PLA CAD mass 320.0 g per pair, 91.3% below historical v0.2.0; no sale/release claim</t>
         </is>
       </c>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">organizer/nameform-bookends/exports/final/nameform-bookends-M-single.3mf</t>
+        </is>
+      </c>
+      <c r="W3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1974,12 +2022,12 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">market_research/bericht-top20-alltags-organizer-kleine-wohnraeume.md</t>
+          <t xml:space="preserve">organizer/shelffit-mini-bins</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research concept</t>
+          <t xml:space="preserve">Local controlled project</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -1987,9 +2035,9 @@
           <t xml:space="preserve">Core</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P0 Idea</t>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 Digital candidate</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -1999,22 +2047,22 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No CAD</t>
+          <t xml:space="preserve">v0.1.0 / 0.1.0-draft.1 CadQuery source; marked STEP/STL and valid one-object DRAFT 3MF; one watertight 210 x 209.5 x 148 mm body; source, mesh, 3MF, reference-layout, optimization and digital watermark checks PASS through interface-validation</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No tests</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">No exact slicer/profile; shelf-clearance/watermark coupons and unchanged pair fit, 1.5 kg load, 100-cycle grip and cleaning tests are NOT RUN</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canonical MM-WM-001-R1 and local source recorded; broader commercial source/component register and product-title review remain open</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low; define non-stacking light-duty limits</t>
+          <t xml:space="preserve">Low to medium; shelf binding, overload, grip/edge and non-stacking misuse require physical qualification</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -2044,24 +2092,39 @@
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approve envelope and interfaces; create common-printer CAD</t>
+          <t xml:space="preserve">Run exact slicer/profile; measure shelf; print clearance/watermark coupons and unchanged pair; complete TP-01 through TP-07</t>
         </is>
       </c>
       <c r="T4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avoid structural or stacking claims in first revision</t>
+          <t xml:space="preserve">DRAFT digital candidate only; non-stacking, open-top reference set for a provisional 420 x 210 x 150 mm shelf; estimated CAD PLA mass 380.2 g per bin; no sale, exact-fit or load claim</t>
+        </is>
+      </c>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">organizer/shelffit-mini-bins/exports/candidate/manufacturing/DRAFT-shelffit-mini-bin-0.1.0-print-two.3mf</t>
+        </is>
+      </c>
+      <c r="W4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T4"/>
+  <autoFilter ref="A1:W4"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:T59"/>
+  <dimension ref="A1:W59"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2078,12 +2141,15 @@
     <col min="12" max="12" width="48" customWidth="1"/>
     <col min="13" max="13" width="48" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="15" max="15" width="37" customWidth="1"/>
     <col min="16" max="16" width="27" customWidth="1"/>
     <col min="17" max="17" width="34" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="48" customWidth="1"/>
     <col min="20" max="20" width="48" customWidth="1"/>
+    <col min="21" max="21" width="46" customWidth="1"/>
+    <col min="22" max="22" width="48" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -2187,6 +2253,21 @@
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model_Status</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model_Evidence_Path</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model_Audit_Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -2211,7 +2292,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">organizer/drawer-inlay</t>
+          <t xml:space="preserve">products/organization-storage/mm-org-001-drawerfit-modular</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -2287,6 +2368,21 @@
       <c r="T2" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Do not call exact-fit or IKEA-compatible until the named drawer revision and measurement tolerance are physically proven</t>
+        </is>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-org-001-drawerfit-modular/DRAFT-schubladen-organizer-R1.3-aspect-safe-030mm/schubladen-organizer/output/DRAFT/DRAFT-R1.3-aspect-safe-030mm-assembly.3mf</t>
+        </is>
+      </c>
+      <c r="W2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2409,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">organizer/nameform-bookends</t>
+          <t xml:space="preserve">products/organization-storage/mm-per-001-nameform-bookends</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -2389,6 +2485,21 @@
       <c r="T3" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">DRAFT digital candidate only; estimated PLA CAD mass 320.0 g per pair, 91.3% below historical v0.2.0; no sale/release claim</t>
+        </is>
+      </c>
+      <c r="U3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-per-001-nameform-bookends/exports/final/nameform-bookends-M-single.3mf</t>
+        </is>
+      </c>
+      <c r="W3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2415,12 +2526,12 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">market_research/bericht-top20-alltags-organizer-kleine-wohnraeume.md</t>
+          <t xml:space="preserve">products/organization-storage/mm-org-002-shelffit-mini-bins</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Research concept</t>
+          <t xml:space="preserve">Local controlled project</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2428,9 +2539,9 @@
           <t xml:space="preserve">Core</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P0 Idea</t>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 Digital candidate</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -2440,22 +2551,22 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No CAD</t>
+          <t xml:space="preserve">v0.1.0 / 0.1.0-draft.1 CadQuery source; marked STEP/STL and valid one-object DRAFT 3MF; one watertight 210 x 209.5 x 148 mm body; source, mesh, 3MF, reference-layout, optimization and digital watermark checks PASS through interface-validation</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No tests</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">No exact slicer/profile; shelf-clearance/watermark coupons and unchanged pair fit, 1.5 kg load, 100-cycle grip and cleaning tests are NOT RUN</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canonical MM-WM-001-R1 and local source recorded; broader commercial source/component register and product-title review remain open</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low; define non-stacking light-duty limits</t>
+          <t xml:space="preserve">Low to medium; shelf binding, overload, grip/edge and non-stacking misuse require physical qualification</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -2485,12 +2596,27 @@
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approve envelope and interfaces; create common-printer CAD</t>
+          <t xml:space="preserve">Run exact slicer/profile; measure shelf; print clearance/watermark coupons and unchanged pair; complete TP-01 through TP-07</t>
         </is>
       </c>
       <c r="T4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avoid structural or stacking claims in first revision</t>
+          <t xml:space="preserve">DRAFT digital candidate only; non-stacking, open-top reference set for a provisional 420 x 210 x 150 mm shelf; estimated CAD PLA mass 380.2 g per bin; no sale, exact-fit or load claim</t>
+        </is>
+      </c>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-org-002-shelffit-mini-bins/exports/candidate/manufacturing/DRAFT-shelffit-mini-bin-0.1.0-print-two.3mf</t>
+        </is>
+      </c>
+      <c r="W4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2643,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">organizer/desk-drawer/modern-carbon-desk-organizer-v1.1.2</t>
+          <t xml:space="preserve">products/organization-storage/mm-org-003-modern-carbon-desk-organizer</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -2542,12 +2668,12 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automated topology/volume/build checks reported PASS; parametric source and exports</t>
+          <t xml:space="preserve">2.0.0-draft.1 compact CadQuery source, JSON parameters, STEP/STL, fit and texture coupons and valid four-item DRAFT 3MF; all five meshes, assembly envelope, build-volume and nominal interface checks PASS through interface-validation</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Experimental; slicer, anti-tip, wear and reproducibility open</t>
+          <t xml:space="preserve">No exact slicer/profile or physical print; coupon fit, drawer cycles, loaded anti-tip, flatness, stack retention and appearance remain open</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -2587,12 +2713,27 @@
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create smaller modular common-printer derivative or qualify as printed-only</t>
+          <t xml:space="preserve">Run exact slicer/profile; print fit and texture coupons; then print unchanged prototype and complete drawer-cycle, loaded anti-tip and appearance checks</t>
         </is>
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current envelope about 320 x 230 x 213.6 mm</t>
+          <t xml:space="preserve">Common-printer derivative now 210 x 190 x 173 mm with two drawers and removable six-bin sorter; DRAFT only; CAD-volume PLA equivalent 1046 g is not slicer deposited mass</t>
+        </is>
+      </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-org-003-modern-carbon-desk-organizer/modern-carbon-desk-organizer-compact-v2.0.0/exports/3mf/DRAFT-MM-ORG-003-modern-carbon-compact-2.0.0-draft.1.3mf</t>
+        </is>
+      </c>
+      <c r="W5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2760,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">organizer/bathroom/premium-parametric-over-toilet-shelf</t>
+          <t xml:space="preserve">products/organization-storage/mm-bth-001-premium-over-toilet-shelf</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -2695,6 +2836,21 @@
       <c r="T6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">680 x 300 x 1650 mm; manufacturing blocked</t>
+        </is>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-bth-001-premium-over-toilet-shelf/output/default/preview/premium_over_toilet_shelf_assembly.stl</t>
+        </is>
+      </c>
+      <c r="W6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2877,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">organizer/bathroom/toilettpaper_stand</t>
+          <t xml:space="preserve">products/organization-storage/mm-bth-002-toilet-paper-fifo-system</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -2797,6 +2953,21 @@
       <c r="T7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Five-roll wall system; legacy GLB is informative only</t>
+        </is>
+      </c>
+      <c r="U7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-bth-002-toilet-paper-fifo-system/2/ZEN_KINTSUGI_WAVE_FIFO_5R_HYBRID_v2.0.0(2)/ZEN_KINTSUGI_WAVE_FIFO_5R_HYBRID_v2.0.0/SIDE_PANEL_A_multicolor.3mf</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2994,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">organizer/nozzle-box/CyberVault-R4-WM1-RELEASE</t>
+          <t xml:space="preserve">products/printer-workshop/mm-mkr-001-cybervault-nozzle-case</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -2899,6 +3070,21 @@
       <c r="T8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Do not infer commercial release from RELEASE directory name</t>
+        </is>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/printer-workshop/mm-mkr-001-cybervault-nozzle-case/CyberVault-R4-WM1-RELEASE/exports/release/cyber_nozzle_case_R4.3mf</t>
+        </is>
+      </c>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -2925,7 +3111,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3d-printing_addons/Kobra3Max_Gehaeuse_CAD_v1/kobra3max_enclosure_project</t>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-001-kobra3max-enclosure</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -3001,6 +3187,21 @@
       <c r="T9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Large hybrid product with wood/acrylic/printed parts</t>
+        </is>
+      </c>
+      <c r="U9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-001-kobra3max-enclosure/kobra3max_enclosure_project/exports/DRAFT/STL/DRAFT_cable_grommet_half_A.stl</t>
+        </is>
+      </c>
+      <c r="W9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3228,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3d-printing_addons/filament_box</t>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-002-filament-drybox-system</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -3103,6 +3304,21 @@
       <c r="T10" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Includes feedthroughs, floor/rod holder, clips and feeder v1-v4</t>
+        </is>
+      </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-002-filament-drybox-system/01_bodenhalter_23_5mm_rohr_2x_drucken.3mf</t>
+        </is>
+      </c>
+      <c r="W10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3345,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fox</t>
+          <t xml:space="preserve">products/art-decor/mm-art-001-fox-mesh-collection</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -3205,6 +3421,21 @@
       <c r="T11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Raw mesh variants are not a product release</t>
+        </is>
+      </c>
+      <c r="U11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-001-fox-mesh-collection/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3462,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opel_Grandland_2018</t>
+          <t xml:space="preserve">products/art-decor/mm-auto-001-opel-grandland-2018-mesh</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -3307,6 +3538,21 @@
       <c r="T12" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Vehicle-branded subject</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-auto-001-opel-grandland-2018-mesh/Untitled.3mf</t>
+        </is>
+      </c>
+      <c r="W12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3579,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plants</t>
+          <t xml:space="preserve">products/art-decor/mm-art-002-plant-mesh</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -3409,6 +3655,21 @@
       <c r="T13" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-002-plant-mesh/plant1_textured_mesh.obj</t>
+        </is>
+      </c>
+      <c r="W13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3696,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unicorn</t>
+          <t xml:space="preserve">products/art-decor/mm-art-003-unicorn-mesh-collection</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -3511,6 +3772,21 @@
       <c r="T14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-003-unicorn-mesh-collection/white_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3813,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">accessoires/honeycomb-hair-clip-r6-final(1)</t>
+          <t xml:space="preserve">products/wearables/mm-acc-001-honeycomb-hair-clip</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -3613,6 +3889,21 @@
       <c r="T15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">FINAL folder name is not commercial approval</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/wearables/mm-acc-001-honeycomb-hair-clip/output-r6-final/extra_large/masculine-honeycomb-hair-clip-r6-extra-large.3mf</t>
+        </is>
+      </c>
+      <c r="W15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3930,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">art/marble_tile</t>
+          <t xml:space="preserve">products/art-decor/mm-dec-001-marble-tile</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -3715,6 +4006,21 @@
       <c r="T16" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Possible decorative-storage surface component</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-dec-001-marble-tile/simple_raw.3mf</t>
+        </is>
+      </c>
+      <c r="W16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3741,7 +4047,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">art/roman_pillar</t>
+          <t xml:space="preserve">products/art-decor/mm-dec-002-roman-pillar</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -3817,6 +4123,21 @@
       <c r="T17" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Could become decor with storage only after redesign</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-dec-002-roman-pillar/mold_negative.3mf</t>
+        </is>
+      </c>
+      <c r="W17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3843,7 +4164,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">barefoot</t>
+          <t xml:space="preserve">products/wearables/mm-sho-001-barefoot-shoe-collection</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -3919,6 +4240,21 @@
       <c r="T18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Several older variants should be consolidated before any future review</t>
+        </is>
+      </c>
+      <c r="U18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/wearables/mm-sho-001-barefoot-shoe-collection/barfussschuh_v6_1_fitfix/v6_sole_left.3mf</t>
+        </is>
+      </c>
+      <c r="W18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3945,7 +4281,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">blasters/rubber_ball_toy_popper</t>
+          <t xml:space="preserve">products/toys-games/mm-toy-001-rubber-ball-toy-popper</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -4021,6 +4357,21 @@
       <c r="T19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Explicit 0.13 J design limit does not equal certification</t>
+        </is>
+      </c>
+      <c r="U19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-toy-001-rubber-ball-toy-popper/rubber_ball_toy_popper/output/toy_popper_assembly_preview_NOT_FOR_PRINT.stl</t>
+        </is>
+      </c>
+      <c r="W19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4398,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">boats/fisher_boat</t>
+          <t xml:space="preserve">products/toys-games/mm-boat-001-fisher-boat</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -4123,6 +4474,21 @@
       <c r="T20" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-boat-001-fisher-boat/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4149,7 +4515,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">boats/fisher_boat_detailed</t>
+          <t xml:space="preserve">products/toys-games/mm-boat-002-fisher-boat-detailed</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -4225,6 +4591,21 @@
       <c r="T21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-boat-002-fisher-boat-detailed/textured_mesh.stl</t>
+        </is>
+      </c>
+      <c r="W21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4632,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">boats/flapping_submarine</t>
+          <t xml:space="preserve">products/toys-games/mm-boat-003-flapping-tail-submarine</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -4327,6 +4708,21 @@
       <c r="T22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Prototype status is explicit</t>
+        </is>
+      </c>
+      <c r="U22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-boat-003-flapping-tail-submarine/exports/stl/ballast_box.stl</t>
+        </is>
+      </c>
+      <c r="W22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4749,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">boats/rocket_boat</t>
+          <t xml:space="preserve">products/toys-games/mm-boat-004-rocket-boat</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -4429,6 +4825,21 @@
       <c r="T23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-boat-004-rocket-boat/textured_mesh.stl</t>
+        </is>
+      </c>
+      <c r="W23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4866,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">boats/toy_boat</t>
+          <t xml:space="preserve">products/toys-games/mm-boat-005-toy-boat</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -4531,6 +4942,21 @@
       <c r="T24" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-boat-005-toy-boat/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4983,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">bowls/sunflower_bowl</t>
+          <t xml:space="preserve">products/home-kitchen-garden/mm-dec-003-sunflower-bowl-tray</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -4633,6 +5059,21 @@
       <c r="T25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Could fit decor-plus-storage strategy after controlled rebuild</t>
+        </is>
+      </c>
+      <c r="U25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/home-kitchen-garden/mm-dec-003-sunflower-bowl-tray/sunflower_bowl/sunflower_bowl.3mf</t>
+        </is>
+      </c>
+      <c r="W25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4659,7 +5100,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">camera_mount/Kobra3Max_Slim_Camera_Arm_v6_FROM_ORIGINAL_MODEL/k3m_camera_arm_v6_from_original_model</t>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-003-kobra3max-camera-arm</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -4735,6 +5176,21 @@
       <c r="T26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Non-external location does not remove provenance block</t>
+        </is>
+      </c>
+      <c r="U26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-003-kobra3max-camera-arm/Kobra3Max_Slim_Camera_Arm_v6_FROM_ORIGINAL_MODEL/k3m_camera_arm_v6_from_original_model/camera_housing_assembly.3mf</t>
+        </is>
+      </c>
+      <c r="W26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4761,7 +5217,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">capybara</t>
+          <t xml:space="preserve">products/art-decor/mm-art-004-capybara-mesh-collection</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -4837,6 +5293,21 @@
       <c r="T27" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-004-capybara-mesh-collection/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4863,7 +5334,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">claw_hammer</t>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-004-claw-hammer-mesh</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -4939,6 +5410,21 @@
       <c r="T28" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/printer-workshop/mm-tool-004-claw-hammer-mesh/textured_mesh.stl</t>
+        </is>
+      </c>
+      <c r="W28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -4965,7 +5451,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">cup</t>
+          <t xml:space="preserve">products/home-kitchen-garden/mm-home-001-cup-and-measuring-spoon</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -5041,6 +5527,21 @@
       <c r="T29" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/home-kitchen-garden/mm-home-001-cup-and-measuring-spoon/becher.3mf</t>
+        </is>
+      </c>
+      <c r="W29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5568,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">dice_tower/unicorn_tower/polygonal-dice-tower-FINAL-release-0.1.2-g1</t>
+          <t xml:space="preserve">products/toys-games/mm-hob-001-polygonal-dice-tower</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -5143,6 +5644,21 @@
       <c r="T30" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Digitally final is not sellable</t>
+        </is>
+      </c>
+      <c r="U30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-hob-001-polygonal-dice-tower/unicorn_tower/polygonal-dice-tower-FINAL-release-0.1.2-g1/dice_tower_project/release-0.1.2-g1/cutters/entry-orientation-clearance-0.1.2-g1.stl</t>
+        </is>
+      </c>
+      <c r="W30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5685,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">fish</t>
+          <t xml:space="preserve">products/art-decor/mm-art-005-fish-mesh-collection</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -5245,6 +5761,21 @@
       <c r="T31" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-005-fish-mesh-collection/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5802,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">garden</t>
+          <t xml:space="preserve">products/home-kitchen-garden/mm-gar-001-rainwater-filter-well</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -5347,6 +5878,21 @@
       <c r="T32" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">R3 about 10.27 kg modeled PETG; both revisions remain draft</t>
+        </is>
+      </c>
+      <c r="U32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/home-kitchen-garden/mm-gar-001-rainwater-filter-well/regenwasser-filterbrunnen_R2_DRAFT/build/draft-r2/preview/components/01_stufe-3-gehaeuse.stl</t>
+        </is>
+      </c>
+      <c r="W32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5919,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">mouse</t>
+          <t xml:space="preserve">products/art-decor/mm-art-006-mouse-mesh-collection</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -5449,6 +5995,21 @@
       <c r="T33" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-006-mouse-mesh-collection/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5475,7 +6036,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzles/parametric_labyrinth_gift_box</t>
+          <t xml:space="preserve">products/toys-games/mm-puz-001-parametric-labyrinth-gift-box</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -5551,6 +6112,21 @@
       <c r="T34" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Good later bridge to personalization</t>
+        </is>
+      </c>
+      <c r="U34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-puz-001-parametric-labyrinth-gift-box/exports/custom/inner.stl</t>
+        </is>
+      </c>
+      <c r="W34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5567,7 +6143,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle Box Concept</t>
+          <t xml:space="preserve">Mystery Puzzle Box</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -5577,12 +6153,12 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzles/puzzle-box</t>
+          <t xml:space="preserve">products/toys-games/mm-puz-002-mystery-puzzle-box</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Local project</t>
+          <t xml:space="preserve">Local controlled project</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -5590,9 +6166,9 @@
           <t xml:space="preserve">Adjacent</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1 Model present</t>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 Digital candidate</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -5602,22 +6178,22 @@
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Design spec/test plan and concept images found; limited exports</t>
+          <t xml:space="preserve">v1.2.0 / 1.2.0-draft.1 CadQuery source; marked body plus lid, slider and return-leaf STEP/STL; valid eight-object DRAFT 3MF; four watertight meshes; source, mesh, 3MF, interface, flexure-screen, procedural-texture and digital-watermark checks PASS through interface-validation</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No tests found</t>
-        </is>
-      </c>
-      <c r="L35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">No exact slicer/profile; slider-fit, PETG leaf, three-latch, 50-cycle, false-release, appearance, cleaning and watermark tests TP-01 through TP-08 are NOT RUN</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canonical MM-WM-001-R1 and local source recorded; broader commercial provenance and product-title review remain open</t>
         </is>
       </c>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium; pinch/jam and contents access</t>
+          <t xml:space="preserve">Medium; pinch/jam, PETG flexure fatigue/creep, loose small parts and failed relock require physical qualification</t>
         </is>
       </c>
       <c r="N35" s="6" t="inlineStr">
@@ -5627,7 +6203,7 @@
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Later after mechanism qualification</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
@@ -5647,12 +6223,27 @@
       </c>
       <c r="S35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complete controlled CAD and digital validation</t>
+          <t xml:space="preserve">Run exact slicer/profile; print fit, flexure and texture/watermark coupons; complete unchanged assembly TP-01 through TP-08</t>
         </is>
       </c>
       <c r="T35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">DRAFT digital candidate only; 250 x 75 x 75 mm; three independent direct latches, 56 recessed vector motifs, estimated combined CAD mass 306.2 g; no reliability, safety or sale claim</t>
+        </is>
+      </c>
+      <c r="U35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/toys-games/mm-puz-002-mystery-puzzle-box/exports/candidate/DRAFT-mystery-puzzle-box-1.2.0-print-set.3mf</t>
+        </is>
+      </c>
+      <c r="W35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5679,7 +6270,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">racehorse</t>
+          <t xml:space="preserve">products/art-decor/mm-art-007-racehorse-mesh-collection</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -5755,6 +6346,21 @@
       <c r="T36" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-007-racehorse-mesh-collection/textured_mesh.3mf</t>
+        </is>
+      </c>
+      <c r="W36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5781,7 +6387,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">sportscar</t>
+          <t xml:space="preserve">products/art-decor/mm-art-008-sports-car-mesh</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -5857,6 +6463,21 @@
       <c r="T37" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-008-sports-car-mesh/textured_mesh (1).glb</t>
+        </is>
+      </c>
+      <c r="W37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5883,7 +6504,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">walls/setzkasten/honeycomb-wood-wall-shelf</t>
+          <t xml:space="preserve">products/organization-storage/mm-wall-001-honeycomb-wood-wall-shelf</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -5959,6 +6580,21 @@
       <c r="T38" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-wall-001-honeycomb-wood-wall-shelf/setzkasten/honeycomb-wood-wall-shelf/generated/bridge-clip.stl</t>
+        </is>
+      </c>
+      <c r="W38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -5985,7 +6621,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">whale</t>
+          <t xml:space="preserve">products/art-decor/mm-art-009-whale-mesh-collection</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -6061,6 +6697,21 @@
       <c r="T39" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — model artifact present</t>
+        </is>
+      </c>
+      <c r="V39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/art-decor/mm-art-009-whale-mesh-collection/textured_mesh.stl</t>
+        </is>
+      </c>
+      <c r="W39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6738,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-001-alex-inventory-workplace-tray</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -6112,12 +6763,12 @@
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Watertight STL and valid STEP; provisional geometry</t>
+          <t xml:space="preserve">0.2.0-draft.1 standalone CadQuery/JSON tray plus 209.30/210.00/210.70 mm full-width gauges; STEP/STL and valid four-object DRAFT 3MF; all meshes, common-220 envelope and provisional interface contract PASS through interface-validation</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No verified furniture-revision fit, slicer, physical or load tests</t>
+          <t xml:space="preserve">No identified furniture revision/measurements, exact slicer/profile or physical gauge/tray/load evidence</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -6157,12 +6808,27 @@
       </c>
       <c r="S40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Measure identified ALEX revision; fit coupon and controlled test print</t>
+          <t xml:space="preserve">Identify and measure the exact furniture revision; print the three width gauges; update envelope if required; then slice and print the unchanged tray</t>
         </is>
       </c>
       <c r="T40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Highest-ranked system-furniture concept</t>
+          <t xml:space="preserve">Measurement pilot only: 210 x 160 x 32 mm tray; ALEX is intended context, not a guaranteed compatibility claim</t>
+        </is>
+      </c>
+      <c r="U40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-001-alex-inventory-workplace-tray/exports/3mf/DRAFT-MM-SYS-001-alex-measurement-pilot-0.2.0-draft.1.3mf</t>
+        </is>
+      </c>
+      <c r="W40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6855,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-002-bror-tool-shadow-tray</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -6214,12 +6880,12 @@
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Watertight STL and valid STEP; provisional geometry</t>
+          <t xml:space="preserve">0.2.0-draft.1 standalone CadQuery/JSON 216 x 180 x 28 mm tray plus 215.30/216.00/216.70 mm gauges; all tool recesses parameterized; STEP/STL and valid four-object DRAFT 3MF; mesh, common-220 and interface checks PASS through interface-validation</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No verified fit, slicer, physical or load tests</t>
+          <t xml:space="preserve">No exact drawer/tool measurements, slicer/profile, gauge print, full print, point-load, cleaning or cycle evidence</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
@@ -6229,7 +6895,7 @@
       </c>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t xml:space="preserve">Medium; drawer fit, tool access and point loads</t>
         </is>
       </c>
       <c r="N41" s="6" t="inlineStr">
@@ -6259,12 +6925,27 @@
       </c>
       <c r="S41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Measure exact BROR drawer/revision and print fit coupon</t>
+          <t xml:space="preserve">Identify and measure exact drawer revision and tools; print width gauges; update envelope/recess clearances; then slice and print unchanged tray</t>
         </is>
       </c>
       <c r="T41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Measurement pilot only; 216 mm width retains 2 mm nominal bed margin per side; BROR/tool fit is not guaranteed</t>
+        </is>
+      </c>
+      <c r="U41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-002-bror-tool-shadow-tray/exports/3mf/DRAFT-MM-SYS-002-bror-measurement-pilot-0.2.0-draft.1.3mf</t>
+        </is>
+      </c>
+      <c r="W41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6972,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-003-pax-asymmetric-accessory-grid</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -6367,6 +7048,21 @@
       <c r="T42" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-003-pax-asymmetric-accessory-grid/exports/stl/03_pax_asymmetric_accessory_grid.stl</t>
+        </is>
+      </c>
+      <c r="W42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6393,7 +7089,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-004-billy-collection-riser</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -6469,6 +7165,21 @@
       <c r="T43" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-004-billy-collection-riser/exports/stl/04_billy_collection_riser.stl</t>
+        </is>
+      </c>
+      <c r="W43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6495,7 +7206,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-005-bror-shadow-board-workflow-cluster</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -6571,6 +7282,21 @@
       <c r="T44" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-005-bror-shadow-board-workflow-cluster/exports/stl/05_bror_shadow_board_workflow_cluster.stl</t>
+        </is>
+      </c>
+      <c r="W44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6597,7 +7323,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-006-kallax-boardgame-matrix</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -6673,6 +7399,21 @@
       <c r="T45" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-006-kallax-boardgame-matrix/exports/stl/06_kallax_boardgame_matrix.stl</t>
+        </is>
+      </c>
+      <c r="W45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6699,7 +7440,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-007-platsa-collection-cells</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -6775,6 +7516,21 @@
       <c r="T46" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-007-platsa-collection-cells/exports/stl/07_platsa_collection_cells.stl</t>
+        </is>
+      </c>
+      <c r="W46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6801,7 +7557,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-008-skadis-precision-tool-cluster</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -6877,6 +7633,21 @@
       <c r="T47" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-008-skadis-precision-tool-cluster/exports/stl/08_skadis_workflow_cluster.stl</t>
+        </is>
+      </c>
+      <c r="W47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -6903,7 +7674,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-009-besta-passive-media-topology</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -6979,6 +7750,21 @@
       <c r="T48" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-009-besta-passive-media-topology/exports/stl/09_besta_media_topology.stl</t>
+        </is>
+      </c>
+      <c r="W48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7005,7 +7791,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-010-omar-ventilated-shelf-deck</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -7081,6 +7867,21 @@
       <c r="T49" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Research recommended as simple MVP only after testing</t>
+        </is>
+      </c>
+      <c r="U49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-010-omar-ventilated-shelf-deck/exports/stl/10_omar_shelf_deck.stl</t>
+        </is>
+      </c>
+      <c r="W49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7908,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-011-boaxel-cleaning-accessory-dock</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -7183,6 +7984,21 @@
       <c r="T50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-011-boaxel-cleaning-accessory-dock/exports/stl/11_boaxel_light_cleaning_docking_rail.stl</t>
+        </is>
+      </c>
+      <c r="W50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7209,7 +8025,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-012-besta-controller-and-media-tray</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -7285,6 +8101,21 @@
       <c r="T51" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-012-besta-controller-and-media-tray/exports/stl/12_besta_controller_media_drawer_tray.stl</t>
+        </is>
+      </c>
+      <c r="W51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7311,7 +8142,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-013-trofast-adult-workshop-insert</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -7387,6 +8218,21 @@
       <c r="T52" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-013-trofast-adult-workshop-insert/exports/stl/13_trofast_adult_workshop_insert.stl</t>
+        </is>
+      </c>
+      <c r="W52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7413,7 +8259,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-014-kallax-creative-material-cassette</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
@@ -7489,6 +8335,21 @@
       <c r="T53" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-014-kallax-creative-material-cassette/exports/stl/14_kallax_creative_material_cassette.stl</t>
+        </is>
+      </c>
+      <c r="W53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7515,7 +8376,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-015-boaxel-basket-microsorter</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -7591,6 +8452,21 @@
       <c r="T54" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-015-boaxel-basket-microsorter/exports/stl/15_boaxel_basket_microsorter.stl</t>
+        </is>
+      </c>
+      <c r="W54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7617,7 +8493,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-016-malm-fold-size-drawer-dividers</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -7693,6 +8569,21 @@
       <c r="T55" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-016-malm-fold-size-drawer-dividers/exports/stl/16_malm_fold_size_dividers.stl</t>
+        </is>
+      </c>
+      <c r="W55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7719,7 +8610,7 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-017-ivar-no-drill-side-inventory-rail</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -7795,6 +8686,21 @@
       <c r="T56" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-017-ivar-no-drill-side-inventory-rail/exports/stl/17_ivar_no_drill_side_inventory_rail.stl</t>
+        </is>
+      </c>
+      <c r="W56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7821,7 +8727,7 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-018-billy-collection-display-matrix</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -7897,6 +8803,21 @@
       <c r="T57" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-018-billy-collection-display-matrix/exports/stl/18_billy_collection_display_matrix.stl</t>
+        </is>
+      </c>
+      <c r="W57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7923,7 +8844,7 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-019-lagkapten-alex-reversible-cable-rail</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
@@ -7999,6 +8920,21 @@
       <c r="T58" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-019-lagkapten-alex-reversible-cable-rail/exports/stl/19_lagkapten_alex_reversible_cable_rail.stl</t>
+        </is>
+      </c>
+      <c r="W58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
@@ -8025,7 +8961,7 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">systemmoebel_top20_cad</t>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-020-lack-leg-two-pocket-mini-dock</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
@@ -8101,11 +9037,26 @@
       <c r="T59" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/furniture-systems/mm-sys-020-lack-leg-two-pocket-mini-dock/exports/stl/20_lack_leg_two_pocket_mini_dock.stl</t>
+        </is>
+      </c>
+      <c r="W59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-26</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T59"/>
+  <autoFilter ref="A1:W59"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -8740,7 +9691,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -9524,14 +10475,14 @@
           <t xml:space="preserve">P0</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In progress</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CadQuery source, marked STEP/STL, valid DRAFT 3MF, 38/38 text sweep and digital checks PASS; exact slicer/profile preflight remains blocked</t>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CadQuery source, marked STEP/STL, valid DRAFT 3MF, 38/38 text sweep and digital checks PASS; exact slicer/profile work continues under BOOK-003</t>
         </is>
       </c>
     </row>
@@ -9680,14 +10631,14 @@
           <t xml:space="preserve">P0</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not started</t>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">requirements and concept approval</t>
+          <t xml:space="preserve">v0.1.0 requirements and generated concept AUTO_APPROVED 2026-08-26 under the user-authorized project policy</t>
         </is>
       </c>
     </row>
@@ -9732,14 +10683,14 @@
           <t xml:space="preserve">P0</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not started</t>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">source/build/digital validation PASS</t>
+          <t xml:space="preserve">0.1.0-draft.1 CadQuery source, marked STEP/STL, valid DRAFT 3MF and frozen aggregate digital validation PASS through interface stage</t>
         </is>
       </c>
     </row>
@@ -9850,32 +10801,32 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAL-001</t>
+          <t xml:space="preserve">DESK-001</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Now</t>
+          <t xml:space="preserve">Next</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Market validation</t>
+          <t xml:space="preserve">Product</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Founder</t>
+          <t xml:space="preserve">CAD owner</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interview 10-15 target users about awkward spaces and current alternatives</t>
+          <t xml:space="preserve">Create common-220 modular derivative of MM-ORG-003 with two drawers, removable six-bin sorter, fit/texture coupons and controlled DRAFT 3MF</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PORT-001</t>
+          <t xml:space="preserve">SHELF-002</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -9888,51 +10839,51 @@
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not started</t>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">notes and synthesized repeated problems without personal-data excess</t>
+          <t xml:space="preserve">2.0.0-draft.1 parametric CadQuery/JSON, STEP/STL and valid four-item 3MF; mesh, envelope and interface gates PASS</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAL-002</t>
+          <t xml:space="preserve">DESK-002</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Now</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Market validation</t>
+          <t xml:space="preserve">Testing</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product owner</t>
+          <t xml:space="preserve">Test owner</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test drawer/shelf measurement guide with 8 users</t>
+          <t xml:space="preserve">Slice MM-ORG-003 Compact, print fit/texture coupons and unchanged prototype, then test cycles, stack retention, loaded anti-tip and appearance</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAL-001</t>
+          <t xml:space="preserve">DESK-001</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-3 d</t>
+          <t xml:space="preserve">3-5 d plus print time</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -9947,14 +10898,14 @@
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">completion time, error/variance and revised guide</t>
+          <t xml:space="preserve">exact slicer report plus unchanged physical test report PASS</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAL-003</t>
+          <t xml:space="preserve">ALEX-001</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -9964,84 +10915,84 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Market validation</t>
+          <t xml:space="preserve">Product</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Founder</t>
+          <t xml:space="preserve">CAD owner</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run honest three-product landing/waitlist and price-preference test</t>
+          <t xml:space="preserve">Convert MM-SYS-001 into a standalone common-220 measurement pilot with parametric tray, width gauges and controlled 3MF</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOOK-001,SHELF-001,DRAW-001</t>
+          <t xml:space="preserve">DESK-001</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 d setup plus observation</t>
+          <t xml:space="preserve">2-3 d</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not started</t>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">qualified interest and file-vs-print evidence; no untrue availability claims</t>
+          <t xml:space="preserve">0.2.0-draft.1 CadQuery/JSON, STEP/STL, three width gauges and valid four-object 3MF; digital gates PASS through interface-validation</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">WEB-001</t>
+          <t xml:space="preserve">ALEX-002</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Now</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering</t>
+          <t xml:space="preserve">Testing</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering lead</t>
+          <t xml:space="preserve">Test owner</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reconcile local website worktree with supplied main commit without losing local edits</t>
+          <t xml:space="preserve">Identify and measure exact furniture revision; print width gauges; update envelope if needed; slice and print unchanged tray</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ALEX-001</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 d</t>
+          <t xml:space="preserve">2-4 d plus print time</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -10051,101 +11002,101 @@
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">clean documented working branch based on approved main</t>
+          <t xml:space="preserve">measurement record, selected gauge and unchanged physical fit/use report PASS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">WEB-002</t>
+          <t xml:space="preserve">BROR-001</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Now</t>
+          <t xml:space="preserve">Next</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering</t>
+          <t xml:space="preserve">Product</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering lead</t>
+          <t xml:space="preserve">CAD owner</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add CI for lint, typecheck, unit, build, Firebase rules and critical E2E; protect main</t>
+          <t xml:space="preserve">Convert MM-SYS-002 into a standalone common-220 tool-tray measurement pilot with parametric recesses, width gauges and controlled 3MF</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">WEB-001</t>
+          <t xml:space="preserve">ALEX-001</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-4 d</t>
+          <t xml:space="preserve">2-3 d</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not started</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">required checks pass on pull request and block failed merge</t>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.2.0-draft.1 CadQuery/JSON, STEP/STL, three gauges and valid four-object 3MF; digital gates PASS through interface-validation</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENV-001</t>
+          <t xml:space="preserve">BROR-002</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Now</t>
+          <t xml:space="preserve">Later</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cloud/Security</t>
+          <t xml:space="preserve">Testing</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering lead</t>
+          <t xml:space="preserve">Test owner</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create separate development, staging and production Firebase/Google Cloud projects and regions</t>
+          <t xml:space="preserve">Measure exact drawer revision and tools; print gauges; update envelope/recess clearance; slice and print unchanged tray</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOV-001,WEB-001</t>
+          <t xml:space="preserve">BROR-001</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-4 d</t>
+          <t xml:space="preserve">2-4 d plus print time</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -10155,49 +11106,49 @@
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">environment inventory, least-privilege identities and deployed rules/indexes</t>
+          <t xml:space="preserve">measurement records, selected gauge and unchanged physical drawer/tool-fit report PASS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEC-001</t>
+          <t xml:space="preserve">VAL-001</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Next</t>
+          <t xml:space="preserve">Now</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cloud/Security</t>
+          <t xml:space="preserve">Market validation</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering lead</t>
+          <t xml:space="preserve">Founder</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configure App Check rollout, secrets, service accounts, signed-URL identity, backup/restore and alarms</t>
+          <t xml:space="preserve">Interview 10-15 target users about awkward spaces and current alternatives</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENV-001</t>
+          <t xml:space="preserve">PORT-001</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3-6 d</t>
+          <t xml:space="preserve">3-5 d</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -10207,49 +11158,49 @@
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">security runbook, restore test and alert evidence</t>
+          <t xml:space="preserve">notes and synthesized repeated problems without personal-data excess</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT-001</t>
+          <t xml:space="preserve">VAL-002</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Next</t>
+          <t xml:space="preserve">Now</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catalog</t>
+          <t xml:space="preserve">Market validation</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publisher + reviewer</t>
+          <t xml:space="preserve">Product owner</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publish first exact P5 product to metriCreate staging through operator approvals and verify shared-ID metriMade eligibility mapping</t>
+          <t xml:space="preserve">Test drawer/shelf measurement guide with 8 users</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DRAW-005 or BOOK-004 or SHELF-004,ENV-001</t>
+          <t xml:space="preserve">VAL-001</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 d</t>
+          <t xml:space="preserve">2-3 d</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -10259,14 +11210,14 @@
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">metriCreate catalog/search/detail/sitemap and any metriMade preview map to the same release manifest/hash</t>
+          <t xml:space="preserve">completion time, error/variance and revised guide</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT-002</t>
+          <t xml:space="preserve">VAL-003</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -10276,32 +11227,32 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catalog</t>
+          <t xml:space="preserve">Market validation</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publisher + reviewer</t>
+          <t xml:space="preserve">Founder</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publish remaining two launch products to metriCreate staging with brand-specific content and no duplicated release records</t>
+          <t xml:space="preserve">Run honest three-product landing/waitlist and price-preference test</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT-001,remaining P5 releases</t>
+          <t xml:space="preserve">BOOK-001,SHELF-001,DRAW-001</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1-2 d</t>
+          <t xml:space="preserve">3 d setup plus observation</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P0</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -10311,14 +11262,14 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">all three exact releases visible in metriCreate staging; eligible metriMade previews preserve IDs/revisions</t>
+          <t xml:space="preserve">qualified interest and file-vs-print evidence; no untrue availability claims</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY-001</t>
+          <t xml:space="preserve">WEB-001</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -10328,27 +11279,27 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Payments/Tax</t>
+          <t xml:space="preserve">Engineering</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finance + engineering</t>
+          <t xml:space="preserve">Engineering lead</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decide Germany digital VAT/tax/accounting treatment and configure Stripe test account</t>
+          <t xml:space="preserve">Reconcile local website worktree with supplied main commit without losing local edits</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOV-001</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-5 d plus advisor lead time</t>
+          <t xml:space="preserve">1 d</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
@@ -10363,39 +11314,39 @@
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">approved tax memo/config and test products/prices</t>
+          <t xml:space="preserve">clean documented working branch based on approved main</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY-002</t>
+          <t xml:space="preserve">WEB-002</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Next</t>
+          <t xml:space="preserve">Now</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Payments/Tax</t>
+          <t xml:space="preserve">Engineering</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering + finance</t>
+          <t xml:space="preserve">Engineering lead</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configure verified webhook, idempotency, retries, refunds, chargeback and accounting export</t>
+          <t xml:space="preserve">Add CI for lint, typecheck, unit, build, Firebase rules and critical E2E; protect main</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY-001,ENV-001</t>
+          <t xml:space="preserve">WEB-001</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -10413,16 +11364,16 @@
           <t xml:space="preserve">Not started</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">positive/duplicate/out-of-order/refund test evidence</t>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">required checks pass on pull request and block failed merge</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LEG-001</t>
+          <t xml:space="preserve">ENV-001</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -10432,27 +11383,27 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legal</t>
+          <t xml:space="preserve">Cloud/Security</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legal owner/counsel</t>
+          <t xml:space="preserve">Engineering lead</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approve operator profile, terms, digital license, privacy, product/safety and Germany country scope</t>
+          <t xml:space="preserve">Create separate development, staging and production Firebase/Google Cloud projects and regions</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOV-001,BRD-001</t>
+          <t xml:space="preserve">GOV-001,WEB-001</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">5-15 d plus counsel lead time</t>
+          <t xml:space="preserve">2-4 d</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
@@ -10467,14 +11418,14 @@
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">versioned signed legal package matching actual providers and products</t>
+          <t xml:space="preserve">environment inventory, least-privilege identities and deployed rules/indexes</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LEG-002</t>
+          <t xml:space="preserve">SEC-001</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -10484,27 +11435,27 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legal/Engineering</t>
+          <t xml:space="preserve">Cloud/Security</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Legal owner + engineering</t>
+          <t xml:space="preserve">Engineering lead</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implement and test electronic withdrawal function, durable confirmations and support email</t>
+          <t xml:space="preserve">Configure App Check rollout, secrets, service accounts, signed-URL identity, backup/restore and alarms</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LEG-001,WEB-001</t>
+          <t xml:space="preserve">ENV-001</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-4 d</t>
+          <t xml:space="preserve">3-6 d</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
@@ -10519,44 +11470,44 @@
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">end-to-end withdrawal submission and confirmation evidence</t>
+          <t xml:space="preserve">security runbook, restore test and alert evidence</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPS-001</t>
+          <t xml:space="preserve">CAT-001</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Now</t>
+          <t xml:space="preserve">Next</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations</t>
+          <t xml:space="preserve">Catalog</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations owner</t>
+          <t xml:space="preserve">Publisher + reviewer</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create support, refund, privacy, rights, safety incident and takedown runbooks with case register</t>
+          <t xml:space="preserve">Publish first exact P5 product to metriCreate staging through operator approvals and verify shared-ID metriMade eligibility mapping</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOV-001</t>
+          <t xml:space="preserve">DRAW-005 or BOOK-004 or SHELF-004,ENV-001</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-3 d</t>
+          <t xml:space="preserve">1 d</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
@@ -10571,14 +11522,14 @@
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">named owner, monitored contact, templates, SLA and tabletop scenario</t>
+          <t xml:space="preserve">metriCreate catalog/search/detail/sitemap and any metriMade preview map to the same release manifest/hash</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPS-002</t>
+          <t xml:space="preserve">CAT-002</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -10588,27 +11539,27 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations</t>
+          <t xml:space="preserve">Catalog</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations + engineering</t>
+          <t xml:space="preserve">Publisher + reviewer</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implement payment/order/entitlement reconciliation and orphaned-storage checks</t>
+          <t xml:space="preserve">Publish remaining two launch products to metriCreate staging with brand-specific content and no duplicated release records</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY-002,ENV-001</t>
+          <t xml:space="preserve">CAT-001,remaining P5 releases</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-4 d</t>
+          <t xml:space="preserve">1-2 d</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
@@ -10623,44 +11574,44 @@
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">scheduled reconciler output and resolved injected discrepancies</t>
+          <t xml:space="preserve">all three exact releases visible in metriCreate staging; eligible metriMade previews preserve IDs/revisions</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">E2E-001</t>
+          <t xml:space="preserve">PAY-001</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Next</t>
+          <t xml:space="preserve">Now</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA</t>
+          <t xml:space="preserve">Payments/Tax</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering + product</t>
+          <t xml:space="preserve">Finance + engineering</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test first metriCreate staging purchase, exact download, expiry, unauthorized access, refund and takedown; verify metriMade-to-metriCreate SKU handoff</t>
+          <t xml:space="preserve">Decide Germany digital VAT/tax/accounting treatment and configure Stripe test account</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT-001,PAY-002,LEG-002,OPS-002</t>
+          <t xml:space="preserve">GOV-001</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-3 d</t>
+          <t xml:space="preserve">2-5 d plus advisor lead time</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -10675,14 +11626,14 @@
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">signed test report for exact commit/config/release and preserved cross-brand product context</t>
+          <t xml:space="preserve">approved tax memo/config and test products/prices</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A11Y-001</t>
+          <t xml:space="preserve">PAY-002</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -10692,22 +11643,22 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA/Legal</t>
+          <t xml:space="preserve">Payments/Tax</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA owner</t>
+          <t xml:space="preserve">Engineering + finance</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complete DE content, browser/mobile and accessibility audit of critical flows</t>
+          <t xml:space="preserve">Configure verified webhook, idempotency, retries, refunds, chargeback and accounting export</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT-002,LEG-001</t>
+          <t xml:space="preserve">PAY-001,ENV-001</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -10717,7 +11668,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P0</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -10727,44 +11678,44 @@
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">documented keyboard/screen-reader/contrast/zoom/browser results</t>
+          <t xml:space="preserve">positive/duplicate/out-of-order/refund test evidence</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAUNCH-001</t>
+          <t xml:space="preserve">LEG-001</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Launch</t>
+          <t xml:space="preserve">Now</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Governance</t>
+          <t xml:space="preserve">Legal</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Founder + release owners</t>
+          <t xml:space="preserve">Legal owner/counsel</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run final launch checklist, rollback/kill-switch drill and written production approval</t>
+          <t xml:space="preserve">Approve operator profile, terms, digital license, privacy, product/safety and Germany country scope</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">E2E-001,A11Y-001,SEC-001,CAT-002</t>
+          <t xml:space="preserve">GOV-001,BRD-001</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1-2 d</t>
+          <t xml:space="preserve">5-15 d plus counsel lead time</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -10779,49 +11730,49 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">all P0 gates PASS; commit/rules/legal/Stripe/releases recorded</t>
+          <t xml:space="preserve">versioned signed legal package matching actual providers and products</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAUNCH-002</t>
+          <t xml:space="preserve">LEG-002</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Launch</t>
+          <t xml:space="preserve">Next</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations</t>
+          <t xml:space="preserve">Legal/Engineering</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations owner</t>
+          <t xml:space="preserve">Legal owner + engineering</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monitor first 10 orders and conduct two-week post-launch review</t>
+          <t xml:space="preserve">Implement and test electronic withdrawal function, durable confirmations and support email</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAUNCH-001</t>
+          <t xml:space="preserve">LEG-001,WEB-001</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ongoing 2 weeks</t>
+          <t xml:space="preserve">2-4 d</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P0</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -10831,24 +11782,24 @@
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">orders reconciled; support/refund/download/product findings reviewed</t>
+          <t xml:space="preserve">end-to-end withdrawal submission and confirmation evidence</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRINT-001</t>
+          <t xml:space="preserve">OPS-001</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Now</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Printed fulfillment</t>
+          <t xml:space="preserve">Operations</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -10858,22 +11809,22 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qualify one premium consumer-ready metriMade standard SKU, capacity, QC traveler, packaging, carrier, returns and insurance</t>
+          <t xml:space="preserve">Create support, refund, privacy, rights, safety incident and takedown runbooks with case register</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAUNCH-002</t>
+          <t xml:space="preserve">GOV-001</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">10-20 d plus pilot</t>
+          <t xml:space="preserve">2-3 d</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P0</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -10883,49 +11834,49 @@
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">signed PRINT_FULFILLMENT_READY evidence and enabled metriMade as-is order for one SKU/country</t>
+          <t xml:space="preserve">named owner, monitored contact, templates, SLA and tabletop scenario</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PACK-001</t>
+          <t xml:space="preserve">OPS-002</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Next</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Packaging/Compliance</t>
+          <t xml:space="preserve">Operations</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations + legal</t>
+          <t xml:space="preserve">Operations + engineering</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complete LUCID/system participation/packaging records for physical pilot</t>
+          <t xml:space="preserve">Implement payment/order/entitlement reconciliation and orphaned-storage checks</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRINT-001</t>
+          <t xml:space="preserve">PAY-002,ENV-001</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2-5 d plus provider lead time</t>
+          <t xml:space="preserve">2-4 d</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P0</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -10935,49 +11886,49 @@
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">registrations/contracts/data process and SKU packaging weights</t>
+          <t xml:space="preserve">scheduled reconciler output and resolved injected discrepancies</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONF-001</t>
+          <t xml:space="preserve">E2E-001</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Later</t>
+          <t xml:space="preserve">Next</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configuration</t>
+          <t xml:space="preserve">QA</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Product + engineering</t>
+          <t xml:space="preserve">Engineering + product</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Design metriCreate server-validated parameterization with immutable generated releases and exact metriMade handoff</t>
+          <t xml:space="preserve">Test first metriCreate staging purchase, exact download, expiry, unauthorized access, refund and takedown; verify metriMade-to-metriCreate SKU handoff</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAUNCH-002,VAL-002</t>
+          <t xml:space="preserve">CAT-001,PAY-002,LEG-002,OPS-002</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">15-30 d</t>
+          <t xml:space="preserve">2-3 d</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P0</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -10987,64 +11938,376 @@
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">cross-domain SKU/revision context, range/negative tests, pricing, review and order/download traceability</t>
+          <t xml:space="preserve">signed test report for exact commit/config/release and preserved cross-brand product context</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">A11Y-001</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Next</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA/Legal</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA owner</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete DE content, browser/mobile and accessibility audit of critical flows</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT-002,LEG-001</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2-4 d</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documented keyboard/screen-reader/contrast/zoom/browser results</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAUNCH-001</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Governance</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Founder + release owners</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run final launch checklist, rollback/kill-switch drill and written production approval</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E2E-001,A11Y-001,SEC-001,CAT-002</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1-2 d</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">all P0 gates PASS; commit/rules/legal/Stripe/releases recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAUNCH-002</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operations</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operations owner</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monitor first 10 orders and conduct two-week post-launch review</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAUNCH-001</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ongoing 2 weeks</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orders reconciled; support/refund/download/product findings reviewed</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRINT-001</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Later</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printed fulfillment</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operations owner</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qualify one premium consumer-ready metriMade standard SKU, capacity, QC traveler, packaging, carrier, returns and insurance</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAUNCH-002</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10-20 d plus pilot</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">signed PRINT_FULFILLMENT_READY evidence and enabled metriMade as-is order for one SKU/country</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PACK-001</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Later</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Packaging/Compliance</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operations + legal</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Complete LUCID/system participation/packaging records for physical pilot</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRINT-001</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2-5 d plus provider lead time</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">registrations/contracts/data process and SKU packaging weights</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONF-001</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Later</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Configuration</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product + engineering</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design metriCreate server-validated parameterization with immutable generated releases and exact metriMade handoff</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAUNCH-002,VAL-002</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15-30 d</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cross-domain SKU/revision context, range/negative tests, pricing, review and order/download traceability</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">EXP-001</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Later</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">International</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Legal + tax + operations</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Create per-country approval matrix before enabling a second country</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">LAUNCH-002</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">5-15 d per country</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">P2</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="I50" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Not started</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr">
+      <c r="J50" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">signed legal/tax/payment/language/support allowlist entry</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J44"/>
+  <autoFilter ref="A1:J50"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
design: add parametric lipstick tube grid
</commit_message>
<xml_diff>
--- a/business/02-portfolio/product-portfolio.xlsx
+++ b/business/02-portfolio/product-portfolio.xlsx
@@ -155,7 +155,7 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
@@ -277,7 +277,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -382,7 +382,7 @@
         </is>
       </c>
       <c r="B18" s="6">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
@@ -14107,7 +14107,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W63"/>
+  <dimension ref="A1:W64"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -21506,8 +21506,125 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PORT-063</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MM-ORG-008</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom Lipstick and Tube Grid</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanity organizer</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-org-008-custom-lipstick-tube-grid</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local controlled project</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Core</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2 Digital candidate</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.1.0-draft.1 parametric CadQuery/JSON candidate; 161 x 107 x 34 mm 4x3 mixed-diameter PETG lattice grid, seven-hole 14-26 mm capture guide, STEP/STL pairs and valid two-object DRAFT 3MF; parameter, mesh, envelope, package and nominal interface checks PASS through interface-validation</t>
+        </is>
+      </c>
+      <c r="K64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No exact slicer/profile; real circular/tapered tube fit, 100 insertion cycles, loaded tipping, cleanability, edge and appearance tests are NOT RUN</t>
+        </is>
+      </c>
+      <c r="L64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local original source; broader commercial source/component register remains open</t>
+        </is>
+      </c>
+      <c r="M64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low; tube mismatch, tip and cleanability require physical qualification</t>
+        </is>
+      </c>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Later</t>
+        </is>
+      </c>
+      <c r="O64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Later after physical qualification</t>
+        </is>
+      </c>
+      <c r="P64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No catalog item</t>
+        </is>
+      </c>
+      <c r="Q64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Research Ideas 100 Wave 1</t>
+        </is>
+      </c>
+      <c r="R64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1 NEXT</t>
+        </is>
+      </c>
+      <c r="S64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Print the diameter guide; capture each real tube; update the JSON list; then print unchanged grid and complete fit, cycle, loaded-tip and cleanability tests</t>
+        </is>
+      </c>
+      <c r="T64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DRAFT storage-only organizer for closed cosmetic containers; no direct formulation contact or travel-retention claim</t>
+        </is>
+      </c>
+      <c r="U64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES — controlled CAD/source + model artifact</t>
+        </is>
+      </c>
+      <c r="V64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">products/organization-storage/mm-org-008-custom-lipstick-tube-grid/exports/3mf/DRAFT-MM-ORG-008-custom-lipstick-tube-grid-0.1.0-draft.1.3mf</t>
+        </is>
+      </c>
+      <c r="W64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W63"/>
+  <autoFilter ref="A1:W64"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -27000,39 +27117,39 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="AU7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOT_STARTED</t>
+      <c r="AU7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MODEL_EXISTS</t>
         </is>
       </c>
       <c r="AV7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MM-ORG-008</t>
         </is>
       </c>
       <c r="AW7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">products/organization-storage/mm-org-008-custom-lipstick-tube-grid</t>
         </is>
       </c>
       <c r="AX7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">products/organization-storage/mm-org-008-custom-lipstick-tube-grid/exports/3mf/DRAFT-MM-ORG-008-custom-lipstick-tube-grid-0.1.0-draft.1.3mf</t>
         </is>
       </c>
       <c r="AY7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">research-backlog</t>
+          <t xml:space="preserve">P2-digital-candidate</t>
         </is>
       </c>
       <c r="AZ7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-08-27</t>
         </is>
       </c>
       <c r="BA7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Parametric 4x3 mixed-diameter PETG lattice grid plus 14-26 mm diameter capture guide; geometry/interface checks pass; exact slicer and physical tube-fit/cycle/tip/cleanability tests remain open.</t>
         </is>
       </c>
       <c r="BB7" s="6" t="inlineStr">

</xml_diff>